<commit_message>
feat: updated pretraining, pretraining results, and setup.bat
</commit_message>
<xml_diff>
--- a/results/results.xlsx
+++ b/results/results.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28925"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\!!Self\Pt1\domain-adapation-main\results\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\nlp-unsupervised-domain-adaptation\results\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{30DE603D-B8FA-403B-ABB3-56195DB6C2A5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9A15EAA6-FA27-42D2-A830-756F312A968D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="13">
   <si>
     <t>SOURCE</t>
   </si>
@@ -58,13 +58,19 @@
   </si>
   <si>
     <t>Pivots</t>
+  </si>
+  <si>
+    <t>NOTES</t>
+  </si>
+  <si>
+    <t>Target keliatan lebih bagus, tapi kalo predict class negatif di target domain jelek dibanding source domain :c</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -72,13 +78,45 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="7">
@@ -171,33 +209,61 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -213,6 +279,55 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>47625</xdr:colOff>
+      <xdr:row>11</xdr:row>
+      <xdr:rowOff>47625</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>189707</xdr:colOff>
+      <xdr:row>38</xdr:row>
+      <xdr:rowOff>65322</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Picture 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{1BD061C5-5F61-46BA-BE72-3A17AC0D13C4}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="654844" y="2524125"/>
+          <a:ext cx="3178176" cy="5161197"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -478,114 +593,170 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="B2:J7"/>
+  <dimension ref="B2:K15"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="36.42578125" customWidth="1"/>
+    <col min="11" max="11" width="47.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B2" s="2" t="s">
+    <row r="2" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B2" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="C2" s="10" t="s">
         <v>0</v>
       </c>
-      <c r="D2" s="4"/>
-      <c r="E2" s="4"/>
-      <c r="F2" s="5"/>
-      <c r="G2" s="8" t="s">
+      <c r="D2" s="11"/>
+      <c r="E2" s="11"/>
+      <c r="F2" s="12"/>
+      <c r="G2" s="14" t="s">
         <v>2</v>
       </c>
-      <c r="H2" s="8"/>
-      <c r="I2" s="8"/>
-      <c r="J2" s="8"/>
-    </row>
-    <row r="3" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="H2" s="15"/>
+      <c r="I2" s="15"/>
+      <c r="J2" s="16"/>
+      <c r="K2" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="3" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B3" s="6"/>
-      <c r="C3" s="7" t="s">
+      <c r="C3" s="13" t="s">
         <v>3</v>
       </c>
-      <c r="D3" s="7" t="s">
+      <c r="D3" s="13" t="s">
         <v>5</v>
       </c>
-      <c r="E3" s="7" t="s">
+      <c r="E3" s="13" t="s">
         <v>6</v>
       </c>
-      <c r="F3" s="7" t="s">
+      <c r="F3" s="13" t="s">
         <v>4</v>
       </c>
-      <c r="G3" s="7" t="s">
+      <c r="G3" s="17" t="s">
         <v>3</v>
       </c>
-      <c r="H3" s="7" t="s">
+      <c r="H3" s="17" t="s">
         <v>5</v>
       </c>
-      <c r="I3" s="7" t="s">
+      <c r="I3" s="17" t="s">
         <v>6</v>
       </c>
-      <c r="J3" s="7" t="s">
+      <c r="J3" s="17" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="4" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B4" s="7" t="s">
+      <c r="K3" s="5"/>
+    </row>
+    <row r="4" spans="2:11" ht="45" x14ac:dyDescent="0.25">
+      <c r="B4" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C4" s="7"/>
-      <c r="D4" s="7"/>
-      <c r="E4" s="7"/>
-      <c r="F4" s="7"/>
-      <c r="G4" s="7"/>
-      <c r="H4" s="7"/>
-      <c r="I4" s="7"/>
-      <c r="J4" s="7"/>
-    </row>
-    <row r="5" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B5" s="7" t="s">
+      <c r="C4" s="7">
+        <v>0.90569999999999995</v>
+      </c>
+      <c r="D4" s="8">
+        <v>0.90920000000000001</v>
+      </c>
+      <c r="E4" s="8">
+        <v>0.90569999999999995</v>
+      </c>
+      <c r="F4" s="8">
+        <v>0.90610000000000002</v>
+      </c>
+      <c r="G4" s="18">
+        <v>0.92110000000000003</v>
+      </c>
+      <c r="H4" s="18">
+        <v>0.92</v>
+      </c>
+      <c r="I4" s="18">
+        <v>0.92110000000000003</v>
+      </c>
+      <c r="J4" s="18">
+        <v>0.92049999999999998</v>
+      </c>
+      <c r="K4" s="3" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="5" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B5" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C5" s="7"/>
-      <c r="D5" s="7"/>
-      <c r="E5" s="7"/>
-      <c r="F5" s="7"/>
-      <c r="G5" s="7"/>
-      <c r="H5" s="7"/>
-      <c r="I5" s="7"/>
-      <c r="J5" s="7"/>
-    </row>
-    <row r="6" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B6" s="7" t="s">
+      <c r="C5" s="8"/>
+      <c r="D5" s="8"/>
+      <c r="E5" s="8"/>
+      <c r="F5" s="8"/>
+      <c r="G5" s="18"/>
+      <c r="H5" s="18"/>
+      <c r="I5" s="18"/>
+      <c r="J5" s="18"/>
+      <c r="K5" s="3"/>
+    </row>
+    <row r="6" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B6" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="C6" s="7"/>
-      <c r="D6" s="7"/>
-      <c r="E6" s="7"/>
-      <c r="F6" s="7"/>
-      <c r="G6" s="7"/>
-      <c r="H6" s="7"/>
-      <c r="I6" s="7"/>
-      <c r="J6" s="7"/>
-    </row>
-    <row r="7" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B7" s="9" t="s">
+      <c r="C6" s="8"/>
+      <c r="D6" s="8"/>
+      <c r="E6" s="8"/>
+      <c r="F6" s="8"/>
+      <c r="G6" s="18"/>
+      <c r="H6" s="18"/>
+      <c r="I6" s="18"/>
+      <c r="J6" s="18"/>
+      <c r="K6" s="3"/>
+    </row>
+    <row r="7" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B7" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="C7" s="1"/>
-      <c r="D7" s="1"/>
-      <c r="E7" s="1"/>
-      <c r="F7" s="1"/>
-      <c r="G7" s="1"/>
-      <c r="H7" s="1"/>
-      <c r="I7" s="1"/>
-      <c r="J7" s="1"/>
+      <c r="C7" s="9"/>
+      <c r="D7" s="9"/>
+      <c r="E7" s="9"/>
+      <c r="F7" s="9"/>
+      <c r="G7" s="19"/>
+      <c r="H7" s="19"/>
+      <c r="I7" s="19"/>
+      <c r="J7" s="19"/>
+      <c r="K7" s="3"/>
+    </row>
+    <row r="8" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="K8" s="2"/>
+    </row>
+    <row r="9" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="K9" s="2"/>
+    </row>
+    <row r="10" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="K10" s="2"/>
+    </row>
+    <row r="11" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B11" t="s">
+        <v>7</v>
+      </c>
+      <c r="K11" s="2"/>
+    </row>
+    <row r="12" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="K12" s="2"/>
+    </row>
+    <row r="13" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="K13" s="2"/>
+    </row>
+    <row r="14" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="K14" s="2"/>
+    </row>
+    <row r="15" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="K15" s="2"/>
     </row>
   </sheetData>
-  <mergeCells count="3">
+  <mergeCells count="4">
     <mergeCell ref="B2:B3"/>
     <mergeCell ref="C2:F2"/>
     <mergeCell ref="G2:J2"/>
+    <mergeCell ref="K2:K3"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Feat: Added adapter result to result excel
</commit_message>
<xml_diff>
--- a/results/results.xlsx
+++ b/results/results.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28925"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\nlp-unsupervised-domain-adaptation\results\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\OV24-2\Folders\Projects\University\Pre-Thesis\nlp-unsupervised-domain-adaptation\results\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9A15EAA6-FA27-42D2-A830-756F312A968D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5CF300D1-D539-44F1-BAB9-788286A7448E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="14">
   <si>
     <t>SOURCE</t>
   </si>
@@ -64,6 +64,12 @@
   </si>
   <si>
     <t>Target keliatan lebih bagus, tapi kalo predict class negatif di target domain jelek dibanding source domain :c</t>
+  </si>
+  <si>
+    <t>Target acc lebih tinggi dari source, tapi class negative di target 
+domain sangat lemah (F1: 0.66) vs positive (F1: 0.94) 
+-&gt; kemungkinan karena imbalance di target test set (6637 pos vs 1032 neg). 
+Overall sedikit di bawah Pretraining, tapi hanya melatih ~3% parameter.</t>
   </si>
 </sst>
 </file>
@@ -209,7 +215,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -220,50 +226,47 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -319,6 +322,50 @@
         <a:xfrm>
           <a:off x="654844" y="2524125"/>
           <a:ext cx="3178176" cy="5161197"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>612913</xdr:colOff>
+      <xdr:row>11</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>565192</xdr:colOff>
+      <xdr:row>38</xdr:row>
+      <xdr:rowOff>49696</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{2D8C8437-A6D3-A8F3-8618-0DB7991928E5}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="4265543" y="2476500"/>
+          <a:ext cx="4242671" cy="5193196"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -601,125 +648,143 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B2" s="4" t="s">
+      <c r="B2" s="10" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="10" t="s">
+      <c r="C2" s="12" t="s">
         <v>0</v>
       </c>
-      <c r="D2" s="11"/>
-      <c r="E2" s="11"/>
-      <c r="F2" s="12"/>
-      <c r="G2" s="14" t="s">
+      <c r="D2" s="13"/>
+      <c r="E2" s="13"/>
+      <c r="F2" s="14"/>
+      <c r="G2" s="15" t="s">
         <v>2</v>
       </c>
-      <c r="H2" s="15"/>
-      <c r="I2" s="15"/>
-      <c r="J2" s="16"/>
-      <c r="K2" s="5" t="s">
+      <c r="H2" s="16"/>
+      <c r="I2" s="16"/>
+      <c r="J2" s="17"/>
+      <c r="K2" s="18" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="3" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B3" s="6"/>
-      <c r="C3" s="13" t="s">
+      <c r="B3" s="11"/>
+      <c r="C3" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="D3" s="13" t="s">
+      <c r="D3" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="E3" s="13" t="s">
+      <c r="E3" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="F3" s="13" t="s">
+      <c r="F3" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="G3" s="17" t="s">
+      <c r="G3" s="7" t="s">
         <v>3</v>
       </c>
-      <c r="H3" s="17" t="s">
+      <c r="H3" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="I3" s="17" t="s">
+      <c r="I3" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="J3" s="17" t="s">
+      <c r="J3" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="K3" s="5"/>
+      <c r="K3" s="18"/>
     </row>
     <row r="4" spans="2:11" ht="45" x14ac:dyDescent="0.25">
       <c r="B4" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C4" s="7">
+      <c r="C4" s="4">
         <v>0.90569999999999995</v>
       </c>
-      <c r="D4" s="8">
+      <c r="D4" s="4">
         <v>0.90920000000000001</v>
       </c>
-      <c r="E4" s="8">
+      <c r="E4" s="4">
         <v>0.90569999999999995</v>
       </c>
-      <c r="F4" s="8">
+      <c r="F4" s="4">
         <v>0.90610000000000002</v>
       </c>
-      <c r="G4" s="18">
+      <c r="G4" s="8">
         <v>0.92110000000000003</v>
       </c>
-      <c r="H4" s="18">
+      <c r="H4" s="8">
         <v>0.92</v>
       </c>
-      <c r="I4" s="18">
+      <c r="I4" s="8">
         <v>0.92110000000000003</v>
       </c>
-      <c r="J4" s="18">
+      <c r="J4" s="8">
         <v>0.92049999999999998</v>
       </c>
       <c r="K4" s="3" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="5" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:11" ht="135" x14ac:dyDescent="0.25">
       <c r="B5" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C5" s="8"/>
-      <c r="D5" s="8"/>
-      <c r="E5" s="8"/>
-      <c r="F5" s="8"/>
-      <c r="G5" s="18"/>
-      <c r="H5" s="18"/>
-      <c r="I5" s="18"/>
-      <c r="J5" s="18"/>
-      <c r="K5" s="3"/>
+      <c r="C5" s="4">
+        <v>0.88759999999999994</v>
+      </c>
+      <c r="D5" s="4">
+        <v>0.89290000000000003</v>
+      </c>
+      <c r="E5" s="4">
+        <v>0.88759999999999994</v>
+      </c>
+      <c r="F5" s="4">
+        <v>0.88800000000000001</v>
+      </c>
+      <c r="G5" s="8">
+        <v>0.90039999999999998</v>
+      </c>
+      <c r="H5" s="8">
+        <v>0.90900000000000003</v>
+      </c>
+      <c r="I5" s="8">
+        <v>0.90039999999999998</v>
+      </c>
+      <c r="J5" s="8">
+        <v>0.90390000000000004</v>
+      </c>
+      <c r="K5" s="3" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="6" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B6" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="C6" s="8"/>
-      <c r="D6" s="8"/>
-      <c r="E6" s="8"/>
-      <c r="F6" s="8"/>
-      <c r="G6" s="18"/>
-      <c r="H6" s="18"/>
-      <c r="I6" s="18"/>
-      <c r="J6" s="18"/>
+      <c r="C6" s="4"/>
+      <c r="D6" s="4"/>
+      <c r="E6" s="4"/>
+      <c r="F6" s="4"/>
+      <c r="G6" s="8"/>
+      <c r="H6" s="8"/>
+      <c r="I6" s="8"/>
+      <c r="J6" s="8"/>
       <c r="K6" s="3"/>
     </row>
     <row r="7" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B7" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="C7" s="9"/>
-      <c r="D7" s="9"/>
-      <c r="E7" s="9"/>
-      <c r="F7" s="9"/>
-      <c r="G7" s="19"/>
-      <c r="H7" s="19"/>
-      <c r="I7" s="19"/>
-      <c r="J7" s="19"/>
+      <c r="C7" s="5"/>
+      <c r="D7" s="5"/>
+      <c r="E7" s="5"/>
+      <c r="F7" s="5"/>
+      <c r="G7" s="9"/>
+      <c r="H7" s="9"/>
+      <c r="I7" s="9"/>
+      <c r="J7" s="9"/>
       <c r="K7" s="3"/>
     </row>
     <row r="8" spans="2:11" x14ac:dyDescent="0.25">
@@ -734,6 +799,9 @@
     <row r="11" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B11" t="s">
         <v>7</v>
+      </c>
+      <c r="E11" t="s">
+        <v>8</v>
       </c>
       <c r="K11" s="2"/>
     </row>

</xml_diff>

<commit_message>
Feat: Fixed adapter results
</commit_message>
<xml_diff>
--- a/results/results.xlsx
+++ b/results/results.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\OV24-2\Folders\Projects\University\Pre-Thesis\nlp-unsupervised-domain-adaptation\results\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5CF300D1-D539-44F1-BAB9-788286A7448E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6C395175-60DD-42FC-8106-C1F607C4D99D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -66,10 +66,10 @@
     <t>Target keliatan lebih bagus, tapi kalo predict class negatif di target domain jelek dibanding source domain :c</t>
   </si>
   <si>
-    <t>Target acc lebih tinggi dari source, tapi class negative di target 
-domain sangat lemah (F1: 0.66) vs positive (F1: 0.94) 
--&gt; kemungkinan karena imbalance di target test set (6637 pos vs 1032 neg). 
-Overall sedikit di bawah Pretraining, tapi hanya melatih ~3% parameter.</t>
+    <t>- Target accuracy lebih tinggi dari source (90.04% vs 88.76%), pola konsisten dengan Pretraining. Namun class negative di target domain sangat lemah (F1: 0.66) vs positive (F1: 0.94)
+-&gt; kemungkinan karena imbalance di target test set (6637 pos vs 1032 neg).
+- MMD loss stabil di 0.382–0.385, domain adapter konvergen tapi gap source-target masih ada.
+Overall sedikit di bawah Pretraining, tapi hanya melatih ~1.83% parameter.</t>
   </si>
 </sst>
 </file>
@@ -215,7 +215,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -266,6 +266,9 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -727,7 +730,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="5" spans="2:11" ht="135" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:11" ht="165" x14ac:dyDescent="0.25">
       <c r="B5" s="1" t="s">
         <v>8</v>
       </c>
@@ -755,7 +758,7 @@
       <c r="J5" s="8">
         <v>0.90390000000000004</v>
       </c>
-      <c r="K5" s="3" t="s">
+      <c r="K5" s="19" t="s">
         <v>13</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Feat: Added Dataset for comparison
</commit_message>
<xml_diff>
--- a/results/results.xlsx
+++ b/results/results.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\OV24-2\Folders\Projects\University\Pre-Thesis\nlp-unsupervised-domain-adaptation\results\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6C395175-60DD-42FC-8106-C1F607C4D99D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{563F5904-4E93-452B-BBBB-465389AE9BB8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -240,6 +240,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -266,9 +269,6 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -651,27 +651,27 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B2" s="10" t="s">
+      <c r="B2" s="11" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="12" t="s">
+      <c r="C2" s="13" t="s">
         <v>0</v>
       </c>
-      <c r="D2" s="13"/>
-      <c r="E2" s="13"/>
-      <c r="F2" s="14"/>
-      <c r="G2" s="15" t="s">
+      <c r="D2" s="14"/>
+      <c r="E2" s="14"/>
+      <c r="F2" s="15"/>
+      <c r="G2" s="16" t="s">
         <v>2</v>
       </c>
-      <c r="H2" s="16"/>
-      <c r="I2" s="16"/>
-      <c r="J2" s="17"/>
-      <c r="K2" s="18" t="s">
+      <c r="H2" s="17"/>
+      <c r="I2" s="17"/>
+      <c r="J2" s="18"/>
+      <c r="K2" s="19" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="3" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B3" s="11"/>
+      <c r="B3" s="12"/>
       <c r="C3" s="6" t="s">
         <v>3</v>
       </c>
@@ -696,7 +696,7 @@
       <c r="J3" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="K3" s="18"/>
+      <c r="K3" s="19"/>
     </row>
     <row r="4" spans="2:11" ht="45" x14ac:dyDescent="0.25">
       <c r="B4" s="1" t="s">
@@ -758,7 +758,7 @@
       <c r="J5" s="8">
         <v>0.90390000000000004</v>
       </c>
-      <c r="K5" s="19" t="s">
+      <c r="K5" s="10" t="s">
         <v>13</v>
       </c>
     </row>

</xml_diff>